<commit_message>
feat: add society-wide member list printing, team profile modals, assigned task reminders, task view tracking, document vault upload notifications, rename support, and fix non-faculty profile completion percentage
</commit_message>
<xml_diff>
--- a/server/Task Assigining.xlsx
+++ b/server/Task Assigining.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,7 +448,7 @@
         <v>6a96f98b7b0aa337fe8ed330</v>
       </c>
       <c r="B2" t="str">
-        <v>(Deleted) x</v>
+        <v>(Deleted - Ongoing) x</v>
       </c>
       <c r="C2" t="str">
         <v>x</v>
@@ -481,10 +481,10 @@
         <v>Deleted on 1/9/2026, 9:45:30 pm</v>
       </c>
       <c r="M2" t="str">
-        <v>Deleted</v>
+        <v>Deleted (Ongoing)</v>
       </c>
       <c r="N2" t="str">
-        <v>Deleted</v>
+        <v>Deleted (Ongoing)</v>
       </c>
     </row>
     <row r="3">
@@ -492,7 +492,7 @@
         <v>6a9722c2ac2b9db4aecd139a</v>
       </c>
       <c r="B3" t="str">
-        <v>(Deleted) tryyy</v>
+        <v>(Deleted - Completed) tryyy</v>
       </c>
       <c r="C3" t="str">
         <v>trytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytrytry</v>
@@ -525,15 +525,370 @@
         <v>Deleted on 2/9/2026, 12:41:00 am</v>
       </c>
       <c r="M3" t="str">
-        <v>Deleted</v>
+        <v>Deleted (Completed)</v>
       </c>
       <c r="N3" t="str">
-        <v>Deleted</v>
+        <v>Deleted (Completed)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>6a983407f429c21fef384829</v>
+      </c>
+      <c r="B4" t="str">
+        <v>(Deleted - Completed) x</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Good morning everyone. Hard work is the true key to success. This competitive world rewards those who combine smart choices with relentless effort. When you face failures, never give up. Keep pushing forward. Your daily hard work will surely pay off and lead you to your dreams</v>
+      </c>
+      <c r="D4" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Gfg Testing Account</v>
+      </c>
+      <c r="G4" t="str">
+        <v>geeksforgeeksbvp@gmail.com</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Om Karakoti</v>
+      </c>
+      <c r="I4" t="str">
+        <v>omkarakoti2008@gmail.com</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2/9/2026, 8:04:47 pm</v>
+      </c>
+      <c r="K4" t="str">
+        <v>No deadline</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Deleted on 2/9/2026, 8:11:32 pm</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Deleted (Completed)</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Deleted (Completed)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>6a9834c4f429c21fef38491b</v>
+      </c>
+      <c r="B5" t="str">
+        <v>(Deleted - Completed) x</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Good morning everyone. Hard work is the true key to success. This competitive world rewards those who combine smart choices with relentless effort. When you face failures, never give up. Keep pushing forward. Your daily hard work will surely pay off and lead you to your dreams</v>
+      </c>
+      <c r="D5" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Gfg Testing Account</v>
+      </c>
+      <c r="G5" t="str">
+        <v>geeksforgeeksbvp@gmail.com</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="I5" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="J5" t="str">
+        <v>2/9/2026, 8:07:56 pm</v>
+      </c>
+      <c r="K5" t="str">
+        <v>3/9/2026, 2:38:00 am</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Deleted on 6/9/2026, 10:10:10 pm</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Deleted (Completed)</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Deleted (Completed)</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>6a9bdb1af8b48c7f112f9423</v>
+      </c>
+      <c r="B6" t="str">
+        <v>To Add pics of remaining Heads into homepage gallery section</v>
+      </c>
+      <c r="C6" t="str" xml:space="preserve">
+        <v xml:space="preserve">This is the cloudinary link :
+https://res.cloudinary.com/duwmby01d/image/upload/v1788098784/IMG-20260830-WA0076_tbvfbj.jpg</v>
+      </c>
+      <c r="D6" t="str">
+        <v>LOW</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="G6" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Nikhil</v>
+      </c>
+      <c r="I6" t="str">
+        <v>nikhilverma897939@gmail.com</v>
+      </c>
+      <c r="J6" t="str">
+        <v>5/9/2026, 2:34:26 pm</v>
+      </c>
+      <c r="K6" t="str">
+        <v>No deadline</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Not completed</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Ongoing</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>6a9bdbf8f8b48c7f112f94d1</v>
+      </c>
+      <c r="B7" t="str">
+        <v>To fix UI of "Assigned by me" , and "All Tasks" tab</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Both UI and breaking in phone so add media queries, since cards of them are going out of screen horizontally and also cards are looking too big in phone screens so fix overall card ui for smaller screens only, else for desktop screen they are perfect.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="G7" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Om Karakoti</v>
+      </c>
+      <c r="I7" t="str">
+        <v>omkarakoti2008@gmail.com</v>
+      </c>
+      <c r="J7" t="str">
+        <v>5/9/2026, 2:38:08 pm</v>
+      </c>
+      <c r="K7" t="str">
+        <v>No deadline</v>
+      </c>
+      <c r="L7" t="str">
+        <v>6/9/2026, 10:08:39 pm</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>6a9bdc3ff8b48c7f112f95bb</v>
+      </c>
+      <c r="B8" t="str">
+        <v>(Deleted - Completed) just for testing</v>
+      </c>
+      <c r="C8" t="str">
+        <v>just for testingjust for testingjust for testingjust for testingjust for testingjust for testingjust for testing</v>
+      </c>
+      <c r="D8" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="G8" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Test member_rechange</v>
+      </c>
+      <c r="I8" t="str">
+        <v>harpreet.02007@gmail.com</v>
+      </c>
+      <c r="J8" t="str">
+        <v>5/9/2026, 2:39:19 pm</v>
+      </c>
+      <c r="K8" t="str">
+        <v>No deadline</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Deleted on 5/9/2026, 2:41:29 pm</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Deleted (Completed)</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Deleted (Completed)</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>6a9bde31f8b48c7f112f971f</v>
+      </c>
+      <c r="B9" t="str">
+        <v>To add more features in task management</v>
+      </c>
+      <c r="C9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1, When someone is assigned with task, with the email notification now onwards let they also receive the site notification
+2, when that person who is assigned with task clicks complete then the person who assigned task should also receive email notification that that x person has completed it.
+3, when on clicking Clicking "Mark Complete" , in a modal add new warning text like if you click without completing your task then rules will be followed and you will not be consdier in any for certificates and still compulsory to particiate without getting certificate and if didnt then will be kicked out of that department</v>
+      </c>
+      <c r="D9" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="G9" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Om Karakoti</v>
+      </c>
+      <c r="I9" t="str">
+        <v>omkarakoti2008@gmail.com</v>
+      </c>
+      <c r="J9" t="str">
+        <v>5/9/2026, 2:47:37 pm</v>
+      </c>
+      <c r="K9" t="str">
+        <v>No deadline</v>
+      </c>
+      <c r="L9" t="str">
+        <v>6/9/2026, 10:21:58 pm</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>6a9d9225647c1b9322bdbc65</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Teams Page images fix</v>
+      </c>
+      <c r="C10" t="str">
+        <v>go to teams page     gfg-bvcoe.in/team     and see the pics of team there, they are stretching which should not be so fix them.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="G10" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Dev Khanna</v>
+      </c>
+      <c r="I10" t="str">
+        <v>devkhanna0607@gmail.com</v>
+      </c>
+      <c r="J10" t="str">
+        <v>6/9/2026, 9:47:41 pm</v>
+      </c>
+      <c r="K10" t="str">
+        <v>10/9/2026, 3:17:00 am</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Not completed</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Ongoing</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>6a9d9f8b79f886cf3a661959</v>
+      </c>
+      <c r="B11" t="str">
+        <v>tryytyrry</v>
+      </c>
+      <c r="C11" t="str">
+        <v>tryytyrrytryytyrrytryytyrry</v>
+      </c>
+      <c r="D11" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Technical</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Dev Malik</v>
+      </c>
+      <c r="G11" t="str">
+        <v>devmalik838400@gmail.com</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Test member_rechange</v>
+      </c>
+      <c r="I11" t="str">
+        <v>harpreet.02007@gmail.com</v>
+      </c>
+      <c r="J11" t="str">
+        <v>6/9/2026, 10:44:51 pm</v>
+      </c>
+      <c r="K11" t="str">
+        <v>12/9/2026, 10:44:00 pm</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Not completed</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Ongoing</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Ongoing</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>